<commit_message>
feat: publish approved Buffer drafts and reconcile platform receipts
</commit_message>
<xml_diff>
--- a/planning/calendrier-publications.xlsx
+++ b/planning/calendrier-publications.xlsx
@@ -43,7 +43,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,16 @@
         <fgColor rgb="00D4F5E3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A9D0F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -78,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +129,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -671,7 +687,7 @@
       <c r="B10" s="10" t="inlineStr">
         <is>
           <t>[Suivi ecee3555f0c8]
-validated
+shared
 I work. I worked.
 I walk. I walked.
 I cook. I cooked.
@@ -1105,9 +1121,9 @@
       <c r="B8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>validated</t>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>shared</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -1139,11 +1155,21 @@
           <t>ecee3555f0c8</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>instagram, tiktok, youtube</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/De3o9Ooj0Wo/
+https://tiktok.com/@englizygo/video/7700139194793889057
+https://www.youtube.com/watch?v=LnhpfHyuG5w</t>
+        </is>
+      </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>Suivi de fabrication ; aucune publication confirmée.
+          <t>Publication terminée confirmée : Buffer : chaque destination au statut sent, avec date et mode automatique.
 Validation : Confirmation explicite utilisateur : Lecture, image et son corrects
 Version 2
 Épisode : content/episodes/2026-10-24_00-09-29-option-1.json</t>

</xml_diff>